<commit_message>
fix(data): use receipt grand total for Domino reference
</commit_message>
<xml_diff>
--- a/jpg-ocr-stat/evaluation/group_03/stat_oracle.xlsx
+++ b/jpg-ocr-stat/evaluation/group_03/stat_oracle.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results" sheetId="1" r:id="Rf8e4d85c71244a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results" sheetId="1" r:id="Recccd540259d4e83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,7 +469,7 @@
         <x:v>2018-03-26</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
-        <x:v>60.60</x:v>
+        <x:v>33.00</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">

</xml_diff>